<commit_message>
mulitline navigation added / frontend slightly broken
</commit_message>
<xml_diff>
--- a/backend/data-filtering/habourline_frompanv_up.xlsx
+++ b/backend/data-filtering/habourline_frompanv_up.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Other Crap\College related crap\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\travel\backend\data-filtering\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3406B24-5BDC-4D7D-9145-7D34D0FDB27B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB3D7AFF-5C40-4292-9813-823EE245BC53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>